<commit_message>
Fix: Correct attendance sheet titles to 'ใบเช็คชื่อ' with clear mai-ek typography and padding
</commit_message>
<xml_diff>
--- a/public/excel/attendance/00_ไฟล์รวมเล่ม_ใบเช็คชื่อทุกฝ่ายและทุกระดับชั้น_ปี69.xlsx
+++ b/public/excel/attendance/00_ไฟล์รวมเล่ม_ใบเช็คชื่อทุกฝ่ายและทุกระดับชั้น_ปี69.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9923" uniqueCount="1320">
   <si>
-    <t>ใบรายชื่อฝ่ายสแตนเชียร์ คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายสแตนเชียร์ คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>ลำดับ</t>
@@ -633,7 +633,7 @@
     <t>เด็กชายจิรสิน ขันทะ</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายขบวนพาเหรด คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายขบวนพาเหรด คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>ม.2/1</t>
@@ -1176,7 +1176,7 @@
     <t>097-021-8357</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายพร็อพและอุปกรณ์ คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายพร็อพและอุปกรณ์ คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>ม.2/3</t>
@@ -1569,7 +1569,7 @@
     <t>นายภูเบศวร์ เล็กไพจิตร</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายเชียร์ลีดเดอร์ คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายเชียร์ลีดเดอร์ คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>35567</t>
@@ -1767,7 +1767,7 @@
     <t>093-976-7913</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายดรัมเมเยอร์ คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายดรัมเมเยอร์ คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>33641</t>
@@ -1845,7 +1845,7 @@
     <t>099-263-2316</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายคัลเลอร์การ์ด คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายคัลเลอร์การ์ด คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34463</t>
@@ -1938,7 +1938,7 @@
     <t>นางสาวกรภัทร์ เลิศรัตนพันธุ์</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายสวัสดิการ คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายสวัสดิการ คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>ม.2/2</t>
@@ -2229,7 +2229,7 @@
     <t>091-969-6155</t>
   </si>
   <si>
-    <t>ใบรายชื่อฝ่ายสตาฟและคณะกรรมการ ม.5 คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อฝ่ายสตาฟและคณะกรรมการ ม.5 คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>32484</t>
@@ -2508,7 +2508,7 @@
     <t>065-854-3845</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬาฟุตบอล คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬาฟุตบอล คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34277</t>
@@ -2781,7 +2781,7 @@
     <t>นายภานุพัฒน์ ลีประเสริฐสุนทร</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬาบาสเกตบอล คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬาบาสเกตบอล คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34283</t>
@@ -2883,7 +2883,7 @@
     <t>082-590-6971</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬาวอลเลย์บอล คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬาวอลเลย์บอล คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34307</t>
@@ -2979,7 +2979,7 @@
     <t>065-003-4526</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬาเซปักตะกร้อ คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬาเซปักตะกร้อ คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34759</t>
@@ -2991,7 +2991,7 @@
     <t>099-405-2582</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬาเปตอง คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬาเปตอง คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34301</t>
@@ -3063,7 +3063,7 @@
     <t>เด็กชายสิรภพ ชุ่มเย็น</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬากรีฑา คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬากรีฑา คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>34271</t>
@@ -3135,7 +3135,7 @@
     <t>นายกษิดิศ ปันทิ</t>
   </si>
   <si>
-    <t>ใบรายชื่อนักกีฬาวิ่ง 16 ขา คณะสีแสด ปี 2569</t>
+    <t>ใบเช็คชื่อนักกีฬาวิ่ง 16 ขา คณะสีแสด ปี 2569</t>
   </si>
   <si>
     <t>33245</t>
@@ -3210,10 +3210,10 @@
     <t>063-861-0700</t>
   </si>
   <si>
-    <t>ใบรายชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 1 ปี 2569</t>
-  </si>
-  <si>
-    <t>ใบรายชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 2 ปี 2569</t>
+    <t>ใบเช็คชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 1 ปี 2569</t>
+  </si>
+  <si>
+    <t>ใบเช็คชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 2 ปี 2569</t>
   </si>
   <si>
     <t>34439</t>
@@ -3285,7 +3285,7 @@
     <t>เด็กหญิงวิรดา -</t>
   </si>
   <si>
-    <t>ใบรายชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 3 ปี 2569</t>
+    <t>ใบเช็คชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 3 ปี 2569</t>
   </si>
   <si>
     <t>33629</t>
@@ -3372,7 +3372,7 @@
     <t>เด็กหญิงศุภัชญา มูลวงษ์</t>
   </si>
   <si>
-    <t>ใบรายชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 4 ปี 2569</t>
+    <t>ใบเช็คชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 4 ปี 2569</t>
   </si>
   <si>
     <t>33150</t>
@@ -3447,7 +3447,7 @@
     <t>นายณนภัส หมื่นนรา</t>
   </si>
   <si>
-    <t>ใบรายชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 5 ปี 2569</t>
+    <t>ใบเช็คชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 5 ปี 2569</t>
   </si>
   <si>
     <t>32846</t>
@@ -3492,7 +3492,7 @@
     <t>นางสาวโอเมียะ -</t>
   </si>
   <si>
-    <t>ใบรายชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 6 ปี 2569</t>
+    <t>ใบเช็คชื่อสมาชิกคณะสีแสด ระดับชั้นมัธยมศึกษาปีที่ 6 ปี 2569</t>
   </si>
   <si>
     <t>31775</t>

</xml_diff>